<commit_message>
Ajout d'un risue AMDEC
</commit_message>
<xml_diff>
--- a/ENR-QUA-10_pilotage_risques_Green_IT.xlsx
+++ b/ENR-QUA-10_pilotage_risques_Green_IT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://facylitiesmultiservices-my.sharepoint.com/personal/paul_pinsolle_fms-ea_com/Documents/Bureau/Gestion-de-projet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A130095D-A5BB-4AB1-ABF4-F9AE60FC36E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{A130095D-A5BB-4AB1-ABF4-F9AE60FC36E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB892B73-4C9D-4BFB-8A01-0BDDAB6B6A06}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-3870" windowWidth="29040" windowHeight="15720" tabRatio="756" firstSheet="1" activeTab="6" xr2:uid="{4DEE9F2C-744A-4F6D-9D3B-5E651EAA2116}"/>
   </bookViews>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="497">
   <si>
     <t>GUIDE</t>
   </si>
@@ -1959,6 +1959,27 @@
   </si>
   <si>
     <t>Risque de dépassement du budget prévisionnel de 60 000 € en raison d'imprévus techniques, d'une mauvaise estimation des coûts ou de dépenbses supplementaires. Un suivi régulier du budget et validation des dépenses obligatoires</t>
+  </si>
+  <si>
+    <t>Retard de la livraison du MVP par rapport à la date prévue</t>
+  </si>
+  <si>
+    <t>Développement logiciel / Planification</t>
+  </si>
+  <si>
+    <t>MVP incomplet lors du salon de la Tech Verte</t>
+  </si>
+  <si>
+    <t>Sous estimation des taches, difficultés techniques, imprévus et dépendances entre les fonctionnalités</t>
+  </si>
+  <si>
+    <t>Diagramme de gantt et suivi régulier de l'avancement</t>
+  </si>
+  <si>
+    <t>Prioriser les fonctionnalités indispensables au MVP, suivre les taches critiques, prévoir une marge pour les imprévus et réaffecter les ressources si nécessaire</t>
+  </si>
+  <si>
+    <t>Le retard de développement pourrait compromettre la présentation du MVP au salon de Tech Verte. La priorisation des fonctionnalités essentielles et le suivi du diagramme de gantt permettront de détecter les dérives et de limiter leur impact</t>
   </si>
 </sst>
 </file>
@@ -40708,43 +40729,73 @@
       </c>
       <c r="AL13" s="81"/>
     </row>
-    <row r="14" spans="1:38" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:38" s="4" customFormat="1" ht="66" x14ac:dyDescent="0.25">
       <c r="B14" s="317" t="s">
         <v>208</v>
       </c>
       <c r="C14" s="318" t="s">
         <v>104</v>
       </c>
-      <c r="D14" s="338"/>
-      <c r="E14" s="320"/>
-      <c r="F14" s="321"/>
-      <c r="G14" s="322"/>
-      <c r="H14" s="323"/>
-      <c r="I14" s="337"/>
-      <c r="J14" s="325"/>
-      <c r="K14" s="326"/>
-      <c r="L14" s="327"/>
-      <c r="M14" s="328" t="str">
+      <c r="D14" s="338" t="s">
+        <v>490</v>
+      </c>
+      <c r="E14" s="320">
+        <v>46300</v>
+      </c>
+      <c r="F14" s="321" t="s">
+        <v>491</v>
+      </c>
+      <c r="G14" s="322" t="s">
+        <v>492</v>
+      </c>
+      <c r="H14" s="323">
+        <v>8</v>
+      </c>
+      <c r="I14" s="337" t="s">
+        <v>493</v>
+      </c>
+      <c r="J14" s="325">
+        <v>6</v>
+      </c>
+      <c r="K14" s="326" t="s">
+        <v>494</v>
+      </c>
+      <c r="L14" s="327">
+        <v>4</v>
+      </c>
+      <c r="M14" s="328">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="N14" s="329" t="str">
+        <v>48</v>
+      </c>
+      <c r="N14" s="329">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="O14" s="318"/>
-      <c r="P14" s="330"/>
-      <c r="Q14" s="331"/>
-      <c r="R14" s="332"/>
-      <c r="S14" s="333"/>
-      <c r="T14" s="334"/>
-      <c r="U14" s="335" t="str">
+        <v>192</v>
+      </c>
+      <c r="O14" s="318" t="s">
+        <v>495</v>
+      </c>
+      <c r="P14" s="330" t="s">
+        <v>480</v>
+      </c>
+      <c r="Q14" s="331">
+        <v>46336</v>
+      </c>
+      <c r="R14" s="332">
+        <v>8</v>
+      </c>
+      <c r="S14" s="333">
+        <v>3</v>
+      </c>
+      <c r="T14" s="334">
+        <v>2</v>
+      </c>
+      <c r="U14" s="335">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="V14" s="329" t="str">
+        <v>24</v>
+      </c>
+      <c r="V14" s="329">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>48</v>
       </c>
       <c r="W14" s="336"/>
       <c r="X14" s="332"/>
@@ -40760,13 +40811,15 @@
       </c>
       <c r="AC14" s="335" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>Low</v>
       </c>
       <c r="AD14" s="329" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-      <c r="AE14" s="336"/>
+        <v>Low</v>
+      </c>
+      <c r="AE14" s="336" t="s">
+        <v>496</v>
+      </c>
       <c r="AL14" s="81"/>
     </row>
     <row r="15" spans="1:38" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Ajout d'un risque AMDEC
</commit_message>
<xml_diff>
--- a/ENR-QUA-10_pilotage_risques_Green_IT.xlsx
+++ b/ENR-QUA-10_pilotage_risques_Green_IT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://facylitiesmultiservices-my.sharepoint.com/personal/paul_pinsolle_fms-ea_com/Documents/Bureau/Gestion-de-projet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{A130095D-A5BB-4AB1-ABF4-F9AE60FC36E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB892B73-4C9D-4BFB-8A01-0BDDAB6B6A06}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{A130095D-A5BB-4AB1-ABF4-F9AE60FC36E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DFD22BA-9D31-4A4A-BDAC-AE4E25DEEFCF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3870" windowWidth="29040" windowHeight="15720" tabRatio="756" firstSheet="1" activeTab="6" xr2:uid="{4DEE9F2C-744A-4F6D-9D3B-5E651EAA2116}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="756" firstSheet="1" activeTab="6" xr2:uid="{4DEE9F2C-744A-4F6D-9D3B-5E651EAA2116}"/>
   </bookViews>
   <sheets>
     <sheet name="Guide utilisateur" sheetId="18" r:id="rId1"/>
@@ -58,7 +58,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="38" r:id="rId13"/>
+    <pivotCache cacheId="0" r:id="rId13"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="512">
   <si>
     <t>GUIDE</t>
   </si>
@@ -1980,6 +1980,51 @@
   </si>
   <si>
     <t>Le retard de développement pourrait compromettre la présentation du MVP au salon de Tech Verte. La priorisation des fonctionnalités essentielles et le suivi du diagramme de gantt permettront de détecter les dérives et de limiter leur impact</t>
+  </si>
+  <si>
+    <t>Infrastructure Cloud insuffisament performante pour supporter l'application</t>
+  </si>
+  <si>
+    <t>Infrastructure informatique/Hébergement Cloud</t>
+  </si>
+  <si>
+    <t>Temps de réponse trop long, indisponibilité de l'application et mauvaise expérience utilisateur lors de la présentation du MVP</t>
+  </si>
+  <si>
+    <t>Ressources serveur sous-dimensionnées, mauvaise configuration, surcharge ou problème réseau</t>
+  </si>
+  <si>
+    <t>Surveillance de l'infrastructure et vérification du fonctionnement de l'environnement Cloud</t>
+  </si>
+  <si>
+    <t>Réaliser des tests de charge, surveiller les performances, dimensionner correctement les ressources Cloud et prévoir une procédure de sauvegarde ou de redémarrage</t>
+  </si>
+  <si>
+    <t>Les performannces insuffisantes de l'infrastructure Cloud pourraient ralentir ou rendre indisponible l'application. Des tests de charge et de surveillance régulière permettront d'anticiper les problèmes et d'adapter les ressources necessaires.</t>
+  </si>
+  <si>
+    <t>Rapports environnementaux contenant des informations ou des méthodes de calcul non conformes aux exigences réglementaires</t>
+  </si>
+  <si>
+    <t>Réglementation environnementale / Expertise carbone</t>
+  </si>
+  <si>
+    <t>Rapports inexacts ou contestables, perte de confiance des utilisateurs et risques juridique pour l'entreprise</t>
+  </si>
+  <si>
+    <t>Mauvaise interprétation de la réglementation, utilisation de méthodes de calcul inadaptées ou absence de vérification des données</t>
+  </si>
+  <si>
+    <t>Vérification des méthodes de calcul et des données par l'experte carbone</t>
+  </si>
+  <si>
+    <t>Faire vérifier les méthodes de calcul et les rapports par Inés, documenter les sources des facteurs d'émission et contrôler la conformité aux référentiels réglementaires applicables</t>
+  </si>
+  <si>
+    <t>Inès avec Alexandre</t>
+  </si>
+  <si>
+    <t>Une non-conformité dezs rapports environnementaux pourrait entrainer des conséquences juridiques et nuire à la crédibilité du projet. La vérification des méthodes de calcul, des sources utilisées et des rapports par l'experte carbone permettra de réduire ce risque.</t>
   </si>
 </sst>
 </file>
@@ -3693,7 +3738,7 @@
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="600">
+  <cellXfs count="599">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
@@ -5039,53 +5084,125 @@
     <xf numFmtId="0" fontId="21" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="5" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="5" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="77" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="76" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="76" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="77" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="63" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="43" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="43" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5121,6 +5238,54 @@
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="76" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="76" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="77" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="77" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="38" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5136,126 +5301,6 @@
     <xf numFmtId="0" fontId="52" fillId="7" borderId="31" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="63" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="43" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="43" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="32" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="42" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="15" borderId="50" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -5265,110 +5310,8 @@
     <xf numFmtId="0" fontId="22" fillId="15" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="59" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="33" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="40" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="32" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="39" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="53" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="36" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="43" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="36" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="43" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="32" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="39" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5408,8 +5351,110 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="32" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="39" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="53" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="36" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="43" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="36" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="43" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="33" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="40" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="32" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="39" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="41" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="35" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="42" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="59" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="15" borderId="50" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -5420,7 +5465,6 @@
     <xf numFmtId="0" fontId="7" fillId="15" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Hyperlink" xfId="5" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -7356,49 +7400,7 @@
           <a:sp3d/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent6">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent6">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent6">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -7458,49 +7460,7 @@
           <a:sp3d/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent5">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent5">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent5">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -7560,49 +7520,7 @@
           <a:sp3d/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent4">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent4">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent4">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -7909,6 +7827,16 @@
             <a:sp3d/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000006-CFB6-48DA-AB22-1F977929EFED}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
@@ -8045,6 +7973,16 @@
             <a:sp3d/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-CFB6-48DA-AB22-1F977929EFED}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
@@ -8181,6 +8119,16 @@
             <a:sp3d/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-CFB6-48DA-AB22-1F977929EFED}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
@@ -32431,7 +32379,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{947756E5-0097-4B26-8C22-90514271E70D}" name="Tableau croisé dynamique1" cacheId="38" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{947756E5-0097-4B26-8C22-90514271E70D}" name="Tableau croisé dynamique1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="A5:D11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="19">
     <pivotField dataField="1" showAll="0"/>
@@ -32561,7 +32509,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE6EABB0-D986-4D1D-8BBE-6DCA42C39CE8}" name="Tableau croisé dynamique3" cacheId="38" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BE6EABB0-D986-4D1D-8BBE-6DCA42C39CE8}" name="Tableau croisé dynamique3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
   <location ref="A53:E58" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="19">
     <pivotField axis="axisPage" dataField="1" multipleItemSelectionAllowed="1" showAll="0" sumSubtotal="1">
@@ -33176,7 +33124,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C5BDCD88-1FEF-402A-B067-BBD6F053C89C}" name="Tableau croisé dynamique2" cacheId="38" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0" chartFormat="24">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C5BDCD88-1FEF-402A-B067-BBD6F053C89C}" name="Tableau croisé dynamique2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0" chartFormat="24">
   <location ref="A28:E31" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="19">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -34173,40 +34121,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="216" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="401"/>
-      <c r="B1" s="493" t="s">
+      <c r="B1" s="517" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="493"/>
-      <c r="D1" s="493"/>
-      <c r="E1" s="493"/>
-      <c r="F1" s="493"/>
-      <c r="G1" s="493"/>
-      <c r="H1" s="493"/>
-      <c r="I1" s="493"/>
+      <c r="C1" s="517"/>
+      <c r="D1" s="517"/>
+      <c r="E1" s="517"/>
+      <c r="F1" s="517"/>
+      <c r="G1" s="517"/>
+      <c r="H1" s="517"/>
+      <c r="I1" s="517"/>
       <c r="J1" s="402"/>
       <c r="K1" s="403"/>
       <c r="L1" s="404"/>
     </row>
     <row r="2" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="211"/>
-      <c r="B2" s="494"/>
-      <c r="C2" s="494"/>
-      <c r="D2" s="494"/>
-      <c r="E2" s="494"/>
-      <c r="F2" s="494"/>
-      <c r="G2" s="494"/>
-      <c r="H2" s="494"/>
-      <c r="I2" s="494"/>
+      <c r="B2" s="518"/>
+      <c r="C2" s="518"/>
+      <c r="D2" s="518"/>
+      <c r="E2" s="518"/>
+      <c r="F2" s="518"/>
+      <c r="G2" s="518"/>
+      <c r="H2" s="518"/>
+      <c r="I2" s="518"/>
       <c r="J2" s="391"/>
       <c r="K2" s="391"/>
       <c r="L2" s="212"/>
     </row>
     <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="211"/>
-      <c r="B3" s="492" t="s">
+      <c r="B3" s="516" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="492"/>
+      <c r="C3" s="516"/>
       <c r="D3" s="443"/>
       <c r="E3" s="443"/>
       <c r="F3" s="443"/>
@@ -34281,10 +34229,10 @@
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="211"/>
-      <c r="B8" s="492" t="s">
+      <c r="B8" s="516" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="492"/>
+      <c r="C8" s="516"/>
       <c r="D8" s="432"/>
       <c r="E8" s="432"/>
       <c r="F8" s="432"/>
@@ -34718,12 +34666,12 @@
       <c r="A34" s="211"/>
       <c r="B34" s="218"/>
       <c r="C34" s="248"/>
-      <c r="D34" s="495" t="s">
+      <c r="D34" s="519" t="s">
         <v>29</v>
       </c>
-      <c r="E34" s="495"/>
-      <c r="F34" s="495"/>
-      <c r="G34" s="495"/>
+      <c r="E34" s="519"/>
+      <c r="F34" s="519"/>
+      <c r="G34" s="519"/>
       <c r="H34" s="216"/>
       <c r="I34" s="216"/>
       <c r="J34" s="216"/>
@@ -35134,16 +35082,16 @@
     <row r="62" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="211"/>
       <c r="B62" s="423"/>
-      <c r="C62" s="491" t="s">
+      <c r="C62" s="515" t="s">
         <v>47</v>
       </c>
-      <c r="D62" s="491"/>
-      <c r="E62" s="491"/>
-      <c r="F62" s="491"/>
-      <c r="G62" s="491"/>
-      <c r="H62" s="491"/>
-      <c r="I62" s="491"/>
-      <c r="J62" s="491"/>
+      <c r="D62" s="515"/>
+      <c r="E62" s="515"/>
+      <c r="F62" s="515"/>
+      <c r="G62" s="515"/>
+      <c r="H62" s="515"/>
+      <c r="I62" s="515"/>
+      <c r="J62" s="515"/>
       <c r="K62" s="426"/>
       <c r="L62" s="212"/>
     </row>
@@ -35666,30 +35614,30 @@
     <row r="97" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="211"/>
       <c r="B97" s="218"/>
-      <c r="C97" s="490" t="s">
+      <c r="C97" s="514" t="s">
         <v>65</v>
       </c>
-      <c r="D97" s="490"/>
-      <c r="E97" s="490"/>
-      <c r="F97" s="490"/>
-      <c r="G97" s="490"/>
-      <c r="H97" s="490"/>
-      <c r="I97" s="490"/>
-      <c r="J97" s="490"/>
+      <c r="D97" s="514"/>
+      <c r="E97" s="514"/>
+      <c r="F97" s="514"/>
+      <c r="G97" s="514"/>
+      <c r="H97" s="514"/>
+      <c r="I97" s="514"/>
+      <c r="J97" s="514"/>
       <c r="K97" s="220"/>
       <c r="L97" s="212"/>
     </row>
     <row r="98" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="211"/>
       <c r="B98" s="218"/>
-      <c r="C98" s="490"/>
-      <c r="D98" s="490"/>
-      <c r="E98" s="490"/>
-      <c r="F98" s="490"/>
-      <c r="G98" s="490"/>
-      <c r="H98" s="490"/>
-      <c r="I98" s="490"/>
-      <c r="J98" s="490"/>
+      <c r="C98" s="514"/>
+      <c r="D98" s="514"/>
+      <c r="E98" s="514"/>
+      <c r="F98" s="514"/>
+      <c r="G98" s="514"/>
+      <c r="H98" s="514"/>
+      <c r="I98" s="514"/>
+      <c r="J98" s="514"/>
       <c r="L98" s="212"/>
     </row>
     <row r="99" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -36069,7 +36017,7 @@
     <row r="3" spans="2:12" ht="25.5" x14ac:dyDescent="0.2">
       <c r="B3" s="110">
         <f ca="1">TODAY()</f>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="E3" s="111" t="s">
         <v>434</v>
@@ -36196,18 +36144,18 @@
     <row r="1" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="211"/>
       <c r="B1" s="211"/>
-      <c r="C1" s="496" t="s">
+      <c r="C1" s="520" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="496"/>
-      <c r="E1" s="496"/>
-      <c r="F1" s="496"/>
-      <c r="G1" s="496"/>
-      <c r="H1" s="496"/>
-      <c r="I1" s="496"/>
-      <c r="J1" s="496"/>
-      <c r="K1" s="496"/>
-      <c r="L1" s="496"/>
+      <c r="D1" s="520"/>
+      <c r="E1" s="520"/>
+      <c r="F1" s="520"/>
+      <c r="G1" s="520"/>
+      <c r="H1" s="520"/>
+      <c r="I1" s="520"/>
+      <c r="J1" s="520"/>
+      <c r="K1" s="520"/>
+      <c r="L1" s="520"/>
       <c r="M1" s="212"/>
     </row>
     <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -36228,35 +36176,35 @@
     <row r="3" spans="1:13" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="211"/>
       <c r="B3" s="221"/>
-      <c r="C3" s="498" t="s">
+      <c r="C3" s="522" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="498"/>
-      <c r="E3" s="498"/>
-      <c r="F3" s="498"/>
-      <c r="G3" s="498"/>
-      <c r="H3" s="498"/>
-      <c r="I3" s="498"/>
-      <c r="J3" s="498"/>
-      <c r="K3" s="498"/>
-      <c r="L3" s="498"/>
+      <c r="D3" s="522"/>
+      <c r="E3" s="522"/>
+      <c r="F3" s="522"/>
+      <c r="G3" s="522"/>
+      <c r="H3" s="522"/>
+      <c r="I3" s="522"/>
+      <c r="J3" s="522"/>
+      <c r="K3" s="522"/>
+      <c r="L3" s="522"/>
       <c r="M3" s="212"/>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="211"/>
       <c r="B4" s="221"/>
-      <c r="C4" s="497" t="s">
+      <c r="C4" s="521" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="497"/>
-      <c r="E4" s="497"/>
-      <c r="F4" s="497"/>
-      <c r="G4" s="497"/>
-      <c r="H4" s="497"/>
-      <c r="I4" s="497"/>
-      <c r="J4" s="497"/>
-      <c r="K4" s="497"/>
-      <c r="L4" s="497"/>
+      <c r="D4" s="521"/>
+      <c r="E4" s="521"/>
+      <c r="F4" s="521"/>
+      <c r="G4" s="521"/>
+      <c r="H4" s="521"/>
+      <c r="I4" s="521"/>
+      <c r="J4" s="521"/>
+      <c r="K4" s="521"/>
+      <c r="L4" s="521"/>
       <c r="M4" s="212"/>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -36294,18 +36242,18 @@
     <row r="7" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="211"/>
       <c r="B7" s="221"/>
-      <c r="C7" s="498" t="s">
+      <c r="C7" s="522" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="498"/>
-      <c r="E7" s="498"/>
-      <c r="F7" s="498"/>
-      <c r="G7" s="498"/>
-      <c r="H7" s="498"/>
-      <c r="I7" s="498"/>
-      <c r="J7" s="498"/>
-      <c r="K7" s="498"/>
-      <c r="L7" s="498"/>
+      <c r="D7" s="522"/>
+      <c r="E7" s="522"/>
+      <c r="F7" s="522"/>
+      <c r="G7" s="522"/>
+      <c r="H7" s="522"/>
+      <c r="I7" s="522"/>
+      <c r="J7" s="522"/>
+      <c r="K7" s="522"/>
+      <c r="L7" s="522"/>
       <c r="M7" s="212"/>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -36396,18 +36344,18 @@
     <row r="25" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="211"/>
       <c r="B25" s="221"/>
-      <c r="C25" s="499" t="s">
+      <c r="C25" s="523" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="499"/>
-      <c r="E25" s="499"/>
-      <c r="F25" s="499"/>
-      <c r="G25" s="499"/>
-      <c r="H25" s="499"/>
-      <c r="I25" s="499"/>
-      <c r="J25" s="499"/>
-      <c r="K25" s="499"/>
-      <c r="L25" s="499"/>
+      <c r="D25" s="523"/>
+      <c r="E25" s="523"/>
+      <c r="F25" s="523"/>
+      <c r="G25" s="523"/>
+      <c r="H25" s="523"/>
+      <c r="I25" s="523"/>
+      <c r="J25" s="523"/>
+      <c r="K25" s="523"/>
+      <c r="L25" s="523"/>
       <c r="M25" s="212"/>
     </row>
     <row r="26" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -36554,18 +36502,18 @@
     <row r="38" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="211"/>
       <c r="B38" s="221"/>
-      <c r="C38" s="500" t="s">
+      <c r="C38" s="524" t="s">
         <v>87</v>
       </c>
-      <c r="D38" s="500"/>
-      <c r="E38" s="500"/>
-      <c r="F38" s="500"/>
-      <c r="G38" s="500"/>
-      <c r="H38" s="500"/>
-      <c r="I38" s="500"/>
-      <c r="J38" s="500"/>
-      <c r="K38" s="500"/>
-      <c r="L38" s="500"/>
+      <c r="D38" s="524"/>
+      <c r="E38" s="524"/>
+      <c r="F38" s="524"/>
+      <c r="G38" s="524"/>
+      <c r="H38" s="524"/>
+      <c r="I38" s="524"/>
+      <c r="J38" s="524"/>
+      <c r="K38" s="524"/>
+      <c r="L38" s="524"/>
       <c r="M38" s="212"/>
     </row>
     <row r="39" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -36604,18 +36552,18 @@
     <row r="42" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="211"/>
       <c r="B42" s="221"/>
-      <c r="C42" s="501" t="s">
+      <c r="C42" s="525" t="s">
         <v>88</v>
       </c>
-      <c r="D42" s="501"/>
-      <c r="E42" s="501"/>
-      <c r="F42" s="501"/>
-      <c r="G42" s="501"/>
-      <c r="H42" s="501"/>
-      <c r="I42" s="501"/>
-      <c r="J42" s="501"/>
-      <c r="K42" s="501"/>
-      <c r="L42" s="501"/>
+      <c r="D42" s="525"/>
+      <c r="E42" s="525"/>
+      <c r="F42" s="525"/>
+      <c r="G42" s="525"/>
+      <c r="H42" s="525"/>
+      <c r="I42" s="525"/>
+      <c r="J42" s="525"/>
+      <c r="K42" s="525"/>
+      <c r="L42" s="525"/>
       <c r="M42" s="212"/>
     </row>
     <row r="43" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -36668,18 +36616,18 @@
     <row r="46" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="211"/>
       <c r="B46" s="221"/>
-      <c r="C46" s="499" t="s">
+      <c r="C46" s="523" t="s">
         <v>91</v>
       </c>
-      <c r="D46" s="499"/>
-      <c r="E46" s="499"/>
-      <c r="F46" s="499"/>
-      <c r="G46" s="499"/>
-      <c r="H46" s="499"/>
-      <c r="I46" s="499"/>
-      <c r="J46" s="499"/>
-      <c r="K46" s="499"/>
-      <c r="L46" s="499"/>
+      <c r="D46" s="523"/>
+      <c r="E46" s="523"/>
+      <c r="F46" s="523"/>
+      <c r="G46" s="523"/>
+      <c r="H46" s="523"/>
+      <c r="I46" s="523"/>
+      <c r="J46" s="523"/>
+      <c r="K46" s="523"/>
+      <c r="L46" s="523"/>
       <c r="M46" s="212"/>
     </row>
     <row r="47" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -36865,33 +36813,33 @@
     <row r="73" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="211"/>
       <c r="B73" s="221"/>
-      <c r="C73" s="499" t="s">
+      <c r="C73" s="523" t="s">
         <v>97</v>
       </c>
-      <c r="D73" s="499"/>
-      <c r="E73" s="499"/>
-      <c r="F73" s="499"/>
-      <c r="G73" s="499"/>
-      <c r="H73" s="499"/>
-      <c r="I73" s="499"/>
-      <c r="J73" s="499"/>
-      <c r="K73" s="499"/>
-      <c r="L73" s="499"/>
+      <c r="D73" s="523"/>
+      <c r="E73" s="523"/>
+      <c r="F73" s="523"/>
+      <c r="G73" s="523"/>
+      <c r="H73" s="523"/>
+      <c r="I73" s="523"/>
+      <c r="J73" s="523"/>
+      <c r="K73" s="523"/>
+      <c r="L73" s="523"/>
       <c r="M73" s="212"/>
     </row>
     <row r="74" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="211"/>
       <c r="B74" s="221"/>
-      <c r="C74" s="499"/>
-      <c r="D74" s="499"/>
-      <c r="E74" s="499"/>
-      <c r="F74" s="499"/>
-      <c r="G74" s="499"/>
-      <c r="H74" s="499"/>
-      <c r="I74" s="499"/>
-      <c r="J74" s="499"/>
-      <c r="K74" s="499"/>
-      <c r="L74" s="499"/>
+      <c r="C74" s="523"/>
+      <c r="D74" s="523"/>
+      <c r="E74" s="523"/>
+      <c r="F74" s="523"/>
+      <c r="G74" s="523"/>
+      <c r="H74" s="523"/>
+      <c r="I74" s="523"/>
+      <c r="J74" s="523"/>
+      <c r="K74" s="523"/>
+      <c r="L74" s="523"/>
       <c r="M74" s="212"/>
     </row>
     <row r="75" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -37594,24 +37542,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="482"/>
-      <c r="B1" s="482"/>
-      <c r="C1" s="482"/>
-      <c r="D1" s="482"/>
-      <c r="E1" s="482"/>
-      <c r="F1" s="482"/>
-      <c r="G1" s="482"/>
-      <c r="H1" s="482"/>
-      <c r="I1" s="482"/>
-      <c r="J1" s="482"/>
-      <c r="K1" s="482"/>
-      <c r="L1" s="482"/>
-      <c r="M1" s="482"/>
-      <c r="N1" s="482"/>
-      <c r="O1" s="482"/>
-      <c r="P1" s="482"/>
-      <c r="Q1" s="482"/>
-      <c r="R1" s="482"/>
+      <c r="A1" s="526"/>
+      <c r="B1" s="526"/>
+      <c r="C1" s="526"/>
+      <c r="D1" s="526"/>
+      <c r="E1" s="526"/>
+      <c r="F1" s="526"/>
+      <c r="G1" s="526"/>
+      <c r="H1" s="526"/>
+      <c r="I1" s="526"/>
+      <c r="J1" s="526"/>
+      <c r="K1" s="526"/>
+      <c r="L1" s="526"/>
+      <c r="M1" s="526"/>
+      <c r="N1" s="526"/>
+      <c r="O1" s="526"/>
+      <c r="P1" s="526"/>
+      <c r="Q1" s="526"/>
+      <c r="R1" s="526"/>
     </row>
     <row r="2" spans="1:26" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="173" t="s">
@@ -37658,10 +37606,10 @@
       <c r="S3" s="172"/>
     </row>
     <row r="4" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="485" t="s">
+      <c r="A4" s="529" t="s">
         <v>173</v>
       </c>
-      <c r="B4" s="486"/>
+      <c r="B4" s="530"/>
       <c r="C4" s="417" t="s">
         <v>174</v>
       </c>
@@ -37678,10 +37626,10 @@
       <c r="P4" s="151"/>
     </row>
     <row r="5" spans="1:26" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="476" t="s">
+      <c r="A5" s="536" t="s">
         <v>175</v>
       </c>
-      <c r="B5" s="477"/>
+      <c r="B5" s="537"/>
       <c r="C5" s="417" t="s">
         <v>439</v>
       </c>
@@ -37704,42 +37652,42 @@
       <c r="P6" s="151"/>
     </row>
     <row r="7" spans="1:26" s="174" customFormat="1" ht="23.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="487" t="s">
+      <c r="A7" s="531" t="s">
         <v>176</v>
       </c>
-      <c r="B7" s="488"/>
-      <c r="C7" s="488"/>
-      <c r="D7" s="488"/>
-      <c r="E7" s="489"/>
-      <c r="F7" s="483" t="s">
+      <c r="B7" s="532"/>
+      <c r="C7" s="532"/>
+      <c r="D7" s="532"/>
+      <c r="E7" s="533"/>
+      <c r="F7" s="527" t="s">
         <v>177</v>
       </c>
-      <c r="G7" s="483"/>
-      <c r="H7" s="483"/>
-      <c r="I7" s="483"/>
-      <c r="J7" s="483"/>
-      <c r="K7" s="483"/>
-      <c r="L7" s="484" t="s">
+      <c r="G7" s="527"/>
+      <c r="H7" s="527"/>
+      <c r="I7" s="527"/>
+      <c r="J7" s="527"/>
+      <c r="K7" s="527"/>
+      <c r="L7" s="528" t="s">
         <v>178</v>
       </c>
-      <c r="M7" s="484"/>
-      <c r="N7" s="484"/>
-      <c r="O7" s="484"/>
-      <c r="P7" s="484"/>
-      <c r="Q7" s="484"/>
-      <c r="R7" s="484"/>
-      <c r="T7" s="478" t="s">
+      <c r="M7" s="528"/>
+      <c r="N7" s="528"/>
+      <c r="O7" s="528"/>
+      <c r="P7" s="528"/>
+      <c r="Q7" s="528"/>
+      <c r="R7" s="528"/>
+      <c r="T7" s="538" t="s">
         <v>179</v>
       </c>
-      <c r="U7" s="479"/>
-      <c r="V7" s="478" t="s">
+      <c r="U7" s="539"/>
+      <c r="V7" s="538" t="s">
         <v>21</v>
       </c>
-      <c r="W7" s="479"/>
-      <c r="X7" s="480" t="s">
+      <c r="W7" s="539"/>
+      <c r="X7" s="540" t="s">
         <v>180</v>
       </c>
-      <c r="Y7" s="481"/>
+      <c r="Y7" s="541"/>
       <c r="Z7" s="383" t="s">
         <v>181</v>
       </c>
@@ -37748,10 +37696,10 @@
       <c r="A8" s="415"/>
       <c r="B8" s="415"/>
       <c r="C8" s="415"/>
-      <c r="D8" s="474" t="s">
+      <c r="D8" s="534" t="s">
         <v>182</v>
       </c>
-      <c r="E8" s="475"/>
+      <c r="E8" s="535"/>
       <c r="F8" s="392"/>
       <c r="G8" s="392"/>
       <c r="H8" s="392"/>
@@ -38156,7 +38104,7 @@
         <v>441</v>
       </c>
       <c r="N15" s="469">
-        <v>46346</v>
+        <v>46285</v>
       </c>
       <c r="O15" s="469" t="s">
         <v>204</v>
@@ -39016,16 +38964,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="T7:U7"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="X7:Y7"/>
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="F7:K7"/>
     <mergeCell ref="L7:R7"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="T7:U7"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="X7:Y7"/>
   </mergeCells>
   <phoneticPr fontId="73" type="noConversion"/>
   <conditionalFormatting sqref="E10:E45">
@@ -39127,17 +39075,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="38.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="502" t="s">
+      <c r="A1" s="542" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="502"/>
-      <c r="C1" s="502"/>
-      <c r="D1" s="502"/>
-      <c r="E1" s="502"/>
-      <c r="F1" s="502"/>
-      <c r="G1" s="502"/>
-      <c r="H1" s="502"/>
-      <c r="I1" s="502"/>
+      <c r="B1" s="542"/>
+      <c r="C1" s="542"/>
+      <c r="D1" s="542"/>
+      <c r="E1" s="542"/>
+      <c r="F1" s="542"/>
+      <c r="G1" s="542"/>
+      <c r="H1" s="542"/>
+      <c r="I1" s="542"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -39191,13 +39139,13 @@
       <c r="A7" s="150" t="s">
         <v>103</v>
       </c>
-      <c r="B7" s="599">
+      <c r="B7">
         <v>1</v>
       </c>
-      <c r="C7" s="599">
+      <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="599">
+      <c r="D7">
         <v>2</v>
       </c>
       <c r="E7"/>
@@ -39208,11 +39156,11 @@
       <c r="A8" s="150" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="599"/>
-      <c r="C8" s="599">
+      <c r="B8"/>
+      <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" s="599">
+      <c r="D8">
         <v>1</v>
       </c>
       <c r="E8"/>
@@ -39223,11 +39171,11 @@
       <c r="A9" s="150" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="599">
+      <c r="B9">
         <v>2</v>
       </c>
-      <c r="C9" s="599"/>
-      <c r="D9" s="599">
+      <c r="C9"/>
+      <c r="D9">
         <v>2</v>
       </c>
       <c r="E9"/>
@@ -39238,11 +39186,11 @@
       <c r="A10" s="150" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="599">
+      <c r="B10">
         <v>1</v>
       </c>
-      <c r="C10" s="599"/>
-      <c r="D10" s="599">
+      <c r="C10"/>
+      <c r="D10">
         <v>1</v>
       </c>
       <c r="E10"/>
@@ -39253,13 +39201,13 @@
       <c r="A11" s="150" t="s">
         <v>221</v>
       </c>
-      <c r="B11" s="599">
+      <c r="B11">
         <v>4</v>
       </c>
-      <c r="C11" s="599">
+      <c r="C11">
         <v>2</v>
       </c>
-      <c r="D11" s="599">
+      <c r="D11">
         <v>6</v>
       </c>
       <c r="E11"/>
@@ -39326,17 +39274,17 @@
       <c r="C22"/>
     </row>
     <row r="24" spans="1:9" ht="38.25" x14ac:dyDescent="0.3">
-      <c r="A24" s="502" t="s">
+      <c r="A24" s="542" t="s">
         <v>222</v>
       </c>
-      <c r="B24" s="502"/>
-      <c r="C24" s="502"/>
-      <c r="D24" s="502"/>
-      <c r="E24" s="502"/>
-      <c r="F24" s="502"/>
-      <c r="G24" s="502"/>
-      <c r="H24" s="502"/>
-      <c r="I24" s="502"/>
+      <c r="B24" s="542"/>
+      <c r="C24" s="542"/>
+      <c r="D24" s="542"/>
+      <c r="E24" s="542"/>
+      <c r="F24" s="542"/>
+      <c r="G24" s="542"/>
+      <c r="H24" s="542"/>
+      <c r="I24" s="542"/>
     </row>
     <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -39390,16 +39338,16 @@
       <c r="A30" t="s">
         <v>440</v>
       </c>
-      <c r="B30" s="599">
+      <c r="B30">
         <v>1</v>
       </c>
-      <c r="C30" s="599">
+      <c r="C30">
         <v>4</v>
       </c>
-      <c r="D30" s="599">
+      <c r="D30">
         <v>1</v>
       </c>
-      <c r="E30" s="599">
+      <c r="E30">
         <v>6</v>
       </c>
       <c r="F30"/>
@@ -39408,16 +39356,16 @@
       <c r="A31" t="s">
         <v>221</v>
       </c>
-      <c r="B31" s="599">
+      <c r="B31">
         <v>1</v>
       </c>
-      <c r="C31" s="599">
+      <c r="C31">
         <v>4</v>
       </c>
-      <c r="D31" s="599">
+      <c r="D31">
         <v>1</v>
       </c>
-      <c r="E31" s="599">
+      <c r="E31">
         <v>6</v>
       </c>
       <c r="F31"/>
@@ -39455,17 +39403,17 @@
       <c r="F35"/>
     </row>
     <row r="47" spans="1:9" ht="38.25" x14ac:dyDescent="0.3">
-      <c r="A47" s="502" t="s">
+      <c r="A47" s="542" t="s">
         <v>224</v>
       </c>
-      <c r="B47" s="502"/>
-      <c r="C47" s="502"/>
-      <c r="D47" s="502"/>
-      <c r="E47" s="502"/>
-      <c r="F47" s="502"/>
-      <c r="G47" s="502"/>
-      <c r="H47" s="502"/>
-      <c r="I47" s="502"/>
+      <c r="B47" s="542"/>
+      <c r="C47" s="542"/>
+      <c r="D47" s="542"/>
+      <c r="E47" s="542"/>
+      <c r="F47" s="542"/>
+      <c r="G47" s="542"/>
+      <c r="H47" s="542"/>
+      <c r="I47" s="542"/>
     </row>
     <row r="49" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
@@ -39539,16 +39487,16 @@
       <c r="A55" s="210" t="s">
         <v>463</v>
       </c>
-      <c r="B55" s="599">
+      <c r="B55">
         <v>1</v>
       </c>
-      <c r="C55" s="599">
+      <c r="C55">
         <v>2</v>
       </c>
-      <c r="D55" s="599">
+      <c r="D55">
         <v>1</v>
       </c>
-      <c r="E55" s="599">
+      <c r="E55">
         <v>4</v>
       </c>
       <c r="F55"/>
@@ -39557,12 +39505,12 @@
       <c r="A56" s="210" t="s">
         <v>464</v>
       </c>
-      <c r="B56" s="599"/>
-      <c r="C56" s="599">
+      <c r="B56"/>
+      <c r="C56">
         <v>1</v>
       </c>
-      <c r="D56" s="599"/>
-      <c r="E56" s="599">
+      <c r="D56"/>
+      <c r="E56">
         <v>1</v>
       </c>
       <c r="F56"/>
@@ -39571,12 +39519,12 @@
       <c r="A57" s="210" t="s">
         <v>465</v>
       </c>
-      <c r="B57" s="599"/>
-      <c r="C57" s="599">
+      <c r="B57"/>
+      <c r="C57">
         <v>1</v>
       </c>
-      <c r="D57" s="599"/>
-      <c r="E57" s="599">
+      <c r="D57"/>
+      <c r="E57">
         <v>1</v>
       </c>
       <c r="F57"/>
@@ -39585,16 +39533,16 @@
       <c r="A58" s="210" t="s">
         <v>221</v>
       </c>
-      <c r="B58" s="599">
+      <c r="B58">
         <v>1</v>
       </c>
-      <c r="C58" s="599">
+      <c r="C58">
         <v>4</v>
       </c>
-      <c r="D58" s="599">
+      <c r="D58">
         <v>1</v>
       </c>
-      <c r="E58" s="599">
+      <c r="E58">
         <v>6</v>
       </c>
       <c r="F58"/>
@@ -39669,18 +39617,18 @@
       <c r="B5" s="382" t="s">
         <v>229</v>
       </c>
-      <c r="C5" s="503" t="s">
+      <c r="C5" s="543" t="s">
         <v>230</v>
       </c>
-      <c r="D5" s="504"/>
-      <c r="E5" s="504" t="s">
+      <c r="D5" s="544"/>
+      <c r="E5" s="544" t="s">
         <v>231</v>
       </c>
-      <c r="F5" s="505"/>
-      <c r="G5" s="503" t="s">
+      <c r="F5" s="545"/>
+      <c r="G5" s="543" t="s">
         <v>232</v>
       </c>
-      <c r="H5" s="506"/>
+      <c r="H5" s="546"/>
     </row>
     <row r="6" spans="1:8" ht="69" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="264">
@@ -39982,16 +39930,16 @@
     <row r="1" spans="1:38" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="S1" s="6"/>
       <c r="Y1" s="6"/>
-      <c r="Z1" s="507" t="str">
+      <c r="Z1" s="511" t="str">
         <f>"0 - "&amp;AE1</f>
         <v>0 - 249</v>
       </c>
-      <c r="AA1" s="507"/>
-      <c r="AB1" s="507" t="s">
+      <c r="AA1" s="511"/>
+      <c r="AB1" s="511" t="s">
         <v>76</v>
       </c>
-      <c r="AC1" s="507"/>
-      <c r="AD1" s="507"/>
+      <c r="AC1" s="511"/>
+      <c r="AD1" s="511"/>
       <c r="AE1" s="3">
         <v>249</v>
       </c>
@@ -40008,16 +39956,16 @@
       </c>
       <c r="S2" s="6"/>
       <c r="Y2" s="6"/>
-      <c r="Z2" s="508" t="str">
+      <c r="Z2" s="512" t="str">
         <f>(AE1+1)&amp;" - "&amp;AE2</f>
         <v>250 - 499</v>
       </c>
-      <c r="AA2" s="508"/>
-      <c r="AB2" s="508" t="s">
+      <c r="AA2" s="512"/>
+      <c r="AB2" s="512" t="s">
         <v>77</v>
       </c>
-      <c r="AC2" s="508"/>
-      <c r="AD2" s="508"/>
+      <c r="AC2" s="512"/>
+      <c r="AD2" s="512"/>
       <c r="AE2" s="3">
         <v>499</v>
       </c>
@@ -40036,7 +39984,7 @@
       <c r="AE3" s="3"/>
     </row>
     <row r="4" spans="1:38" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="539" t="s">
+      <c r="B4" s="476" t="s">
         <v>293</v>
       </c>
       <c r="C4" s="277"/>
@@ -40064,16 +40012,16 @@
       <c r="W4" s="281"/>
       <c r="X4" s="281"/>
       <c r="Y4" s="282"/>
-      <c r="Z4" s="509" t="str">
+      <c r="Z4" s="513" t="str">
         <f>(AE2+1)&amp;" - "&amp;AE4</f>
         <v>500 - 749</v>
       </c>
-      <c r="AA4" s="509"/>
-      <c r="AB4" s="509" t="s">
+      <c r="AA4" s="513"/>
+      <c r="AB4" s="513" t="s">
         <v>78</v>
       </c>
-      <c r="AC4" s="509"/>
-      <c r="AD4" s="509"/>
+      <c r="AC4" s="513"/>
+      <c r="AD4" s="513"/>
       <c r="AE4" s="283">
         <v>749</v>
       </c>
@@ -40082,7 +40030,7 @@
       </c>
     </row>
     <row r="5" spans="1:38" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="540"/>
+      <c r="B5" s="477"/>
       <c r="C5" s="284"/>
       <c r="D5" s="285" t="s">
         <v>295</v>
@@ -40110,16 +40058,16 @@
       <c r="W5" s="288"/>
       <c r="X5" s="288"/>
       <c r="Y5" s="282"/>
-      <c r="Z5" s="510" t="str">
+      <c r="Z5" s="488" t="str">
         <f>(AE4+1)&amp;" - "&amp;AE5</f>
         <v>750 - 1000</v>
       </c>
-      <c r="AA5" s="510"/>
-      <c r="AB5" s="510" t="s">
+      <c r="AA5" s="488"/>
+      <c r="AB5" s="488" t="s">
         <v>79</v>
       </c>
-      <c r="AC5" s="510"/>
-      <c r="AD5" s="510"/>
+      <c r="AC5" s="488"/>
+      <c r="AD5" s="488"/>
       <c r="AE5" s="283">
         <v>1000</v>
       </c>
@@ -40206,10 +40154,10 @@
       <c r="Z7" s="294"/>
       <c r="AA7" s="294"/>
       <c r="AB7" s="300"/>
-      <c r="AC7" s="511" t="s">
+      <c r="AC7" s="489" t="s">
         <v>304</v>
       </c>
-      <c r="AD7" s="512"/>
+      <c r="AD7" s="490"/>
       <c r="AE7" s="301"/>
       <c r="AF7" s="375">
         <v>6</v>
@@ -40312,88 +40260,88 @@
       </c>
     </row>
     <row r="9" spans="1:38" s="60" customFormat="1" ht="115.5" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="513"/>
-      <c r="C9" s="515" t="s">
+      <c r="B9" s="491"/>
+      <c r="C9" s="493" t="s">
         <v>324</v>
       </c>
-      <c r="D9" s="517" t="s">
+      <c r="D9" s="495" t="s">
         <v>325</v>
       </c>
-      <c r="E9" s="519" t="s">
+      <c r="E9" s="497" t="s">
         <v>326</v>
       </c>
-      <c r="F9" s="521" t="s">
+      <c r="F9" s="499" t="s">
         <v>327</v>
       </c>
-      <c r="G9" s="523" t="s">
+      <c r="G9" s="501" t="s">
         <v>328</v>
       </c>
       <c r="H9" s="313" t="s">
         <v>329</v>
       </c>
-      <c r="I9" s="525" t="s">
+      <c r="I9" s="503" t="s">
         <v>330</v>
       </c>
       <c r="J9" s="314" t="s">
         <v>331</v>
       </c>
-      <c r="K9" s="545" t="s">
+      <c r="K9" s="486" t="s">
         <v>332</v>
       </c>
       <c r="L9" s="315" t="s">
         <v>333</v>
       </c>
-      <c r="M9" s="527" t="s">
+      <c r="M9" s="480" t="s">
         <v>334</v>
       </c>
-      <c r="N9" s="529" t="s">
+      <c r="N9" s="482" t="s">
         <v>335</v>
       </c>
-      <c r="O9" s="531" t="s">
+      <c r="O9" s="505" t="s">
         <v>336</v>
       </c>
-      <c r="P9" s="519" t="s">
+      <c r="P9" s="497" t="s">
         <v>337</v>
       </c>
-      <c r="Q9" s="533" t="s">
+      <c r="Q9" s="507" t="s">
         <v>338</v>
       </c>
-      <c r="R9" s="541" t="s">
+      <c r="R9" s="478" t="s">
         <v>329</v>
       </c>
-      <c r="S9" s="527" t="s">
+      <c r="S9" s="480" t="s">
         <v>331</v>
       </c>
-      <c r="T9" s="529" t="s">
+      <c r="T9" s="482" t="s">
         <v>333</v>
       </c>
-      <c r="U9" s="541" t="s">
+      <c r="U9" s="478" t="s">
         <v>334</v>
       </c>
-      <c r="V9" s="543"/>
-      <c r="W9" s="537" t="s">
+      <c r="V9" s="484"/>
+      <c r="W9" s="474" t="s">
         <v>339</v>
       </c>
-      <c r="X9" s="541" t="s">
+      <c r="X9" s="478" t="s">
         <v>329</v>
       </c>
-      <c r="Y9" s="527" t="s">
+      <c r="Y9" s="480" t="s">
         <v>331</v>
       </c>
-      <c r="Z9" s="529" t="s">
+      <c r="Z9" s="482" t="s">
         <v>333</v>
       </c>
-      <c r="AA9" s="541" t="s">
+      <c r="AA9" s="478" t="s">
         <v>334</v>
       </c>
-      <c r="AB9" s="543"/>
-      <c r="AC9" s="541" t="s">
+      <c r="AB9" s="484"/>
+      <c r="AC9" s="478" t="s">
         <v>322</v>
       </c>
-      <c r="AD9" s="535" t="s">
+      <c r="AD9" s="509" t="s">
         <v>340</v>
       </c>
-      <c r="AE9" s="537"/>
+      <c r="AE9" s="474"/>
       <c r="AF9" s="2">
         <v>8</v>
       </c>
@@ -40403,42 +40351,42 @@
       <c r="AJ9" s="2"/>
     </row>
     <row r="10" spans="1:38" s="60" customFormat="1" ht="83.25" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="514"/>
-      <c r="C10" s="516"/>
-      <c r="D10" s="518"/>
-      <c r="E10" s="520"/>
-      <c r="F10" s="522"/>
-      <c r="G10" s="524"/>
+      <c r="B10" s="492"/>
+      <c r="C10" s="494"/>
+      <c r="D10" s="496"/>
+      <c r="E10" s="498"/>
+      <c r="F10" s="500"/>
+      <c r="G10" s="502"/>
       <c r="H10" s="316" t="s">
         <v>341</v>
       </c>
-      <c r="I10" s="526"/>
+      <c r="I10" s="504"/>
       <c r="J10" s="316" t="s">
         <v>341</v>
       </c>
-      <c r="K10" s="546"/>
+      <c r="K10" s="487"/>
       <c r="L10" s="316" t="s">
         <v>341</v>
       </c>
-      <c r="M10" s="528"/>
-      <c r="N10" s="530"/>
-      <c r="O10" s="532"/>
-      <c r="P10" s="520"/>
-      <c r="Q10" s="534"/>
-      <c r="R10" s="542"/>
-      <c r="S10" s="528"/>
-      <c r="T10" s="530"/>
-      <c r="U10" s="542"/>
-      <c r="V10" s="544"/>
-      <c r="W10" s="538"/>
-      <c r="X10" s="542"/>
-      <c r="Y10" s="528"/>
-      <c r="Z10" s="530"/>
-      <c r="AA10" s="542"/>
-      <c r="AB10" s="544"/>
-      <c r="AC10" s="542"/>
-      <c r="AD10" s="536"/>
-      <c r="AE10" s="538"/>
+      <c r="M10" s="481"/>
+      <c r="N10" s="483"/>
+      <c r="O10" s="506"/>
+      <c r="P10" s="498"/>
+      <c r="Q10" s="508"/>
+      <c r="R10" s="479"/>
+      <c r="S10" s="481"/>
+      <c r="T10" s="483"/>
+      <c r="U10" s="479"/>
+      <c r="V10" s="485"/>
+      <c r="W10" s="475"/>
+      <c r="X10" s="479"/>
+      <c r="Y10" s="481"/>
+      <c r="Z10" s="483"/>
+      <c r="AA10" s="479"/>
+      <c r="AB10" s="485"/>
+      <c r="AC10" s="479"/>
+      <c r="AD10" s="510"/>
+      <c r="AE10" s="475"/>
       <c r="AF10" s="2">
         <v>9</v>
       </c>
@@ -40624,7 +40572,7 @@
         <v>-</v>
       </c>
       <c r="AC12" s="335" t="str">
-        <f t="shared" ref="AC11:AC38" si="7">IF(AB12="-",AD12,IF(AB12&gt;$AE$4,"Very High",IF(AB12&gt;$AE$2,"High",IF(AB12&gt;$AE$1,"Medium",IF(AB12&gt;0,"Low","")))))</f>
+        <f t="shared" ref="AC12:AC38" si="7">IF(AB12="-",AD12,IF(AB12&gt;$AE$4,"Very High",IF(AB12&gt;$AE$2,"High",IF(AB12&gt;$AE$1,"Medium",IF(AB12&gt;0,"Low","")))))</f>
         <v>Low</v>
       </c>
       <c r="AD12" s="329" t="str">
@@ -40822,43 +40770,73 @@
       </c>
       <c r="AL14" s="81"/>
     </row>
-    <row r="15" spans="1:38" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:38" s="4" customFormat="1" ht="82.5" x14ac:dyDescent="0.25">
       <c r="B15" s="317" t="s">
         <v>209</v>
       </c>
       <c r="C15" s="318" t="s">
         <v>104</v>
       </c>
-      <c r="D15" s="338"/>
-      <c r="E15" s="320"/>
-      <c r="F15" s="321"/>
-      <c r="G15" s="322"/>
-      <c r="H15" s="323"/>
-      <c r="I15" s="324"/>
-      <c r="J15" s="325"/>
-      <c r="K15" s="326"/>
-      <c r="L15" s="327"/>
-      <c r="M15" s="328" t="str">
+      <c r="D15" s="338" t="s">
+        <v>497</v>
+      </c>
+      <c r="E15" s="320">
+        <v>46336</v>
+      </c>
+      <c r="F15" s="321" t="s">
+        <v>498</v>
+      </c>
+      <c r="G15" s="322" t="s">
+        <v>499</v>
+      </c>
+      <c r="H15" s="323">
+        <v>7</v>
+      </c>
+      <c r="I15" s="324" t="s">
+        <v>500</v>
+      </c>
+      <c r="J15" s="325">
+        <v>4</v>
+      </c>
+      <c r="K15" s="326" t="s">
+        <v>501</v>
+      </c>
+      <c r="L15" s="327">
+        <v>5</v>
+      </c>
+      <c r="M15" s="328">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="N15" s="329" t="str">
+        <v>28</v>
+      </c>
+      <c r="N15" s="329">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="O15" s="318"/>
-      <c r="P15" s="330"/>
-      <c r="Q15" s="331"/>
-      <c r="R15" s="332"/>
-      <c r="S15" s="333"/>
-      <c r="T15" s="334"/>
-      <c r="U15" s="335" t="str">
+        <v>140</v>
+      </c>
+      <c r="O15" s="318" t="s">
+        <v>502</v>
+      </c>
+      <c r="P15" s="330" t="s">
+        <v>452</v>
+      </c>
+      <c r="Q15" s="331">
+        <v>46349</v>
+      </c>
+      <c r="R15" s="332">
+        <v>7</v>
+      </c>
+      <c r="S15" s="333">
+        <v>2</v>
+      </c>
+      <c r="T15" s="334">
+        <v>3</v>
+      </c>
+      <c r="U15" s="335">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="V15" s="329" t="str">
+        <v>14</v>
+      </c>
+      <c r="V15" s="329">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>42</v>
       </c>
       <c r="W15" s="336"/>
       <c r="X15" s="332"/>
@@ -40874,52 +40852,84 @@
       </c>
       <c r="AC15" s="335" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>Low</v>
       </c>
       <c r="AD15" s="329" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-      <c r="AE15" s="336"/>
+        <v>Low</v>
+      </c>
+      <c r="AE15" s="336" t="s">
+        <v>503</v>
+      </c>
       <c r="AL15" s="81"/>
     </row>
-    <row r="16" spans="1:38" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:38" s="4" customFormat="1" ht="82.5" x14ac:dyDescent="0.25">
       <c r="B16" s="317" t="s">
         <v>451</v>
       </c>
       <c r="C16" s="318" t="s">
         <v>103</v>
       </c>
-      <c r="D16" s="338"/>
-      <c r="E16" s="320"/>
-      <c r="F16" s="321"/>
-      <c r="G16" s="322"/>
-      <c r="H16" s="323"/>
-      <c r="I16" s="324"/>
-      <c r="J16" s="325"/>
-      <c r="K16" s="326"/>
-      <c r="L16" s="327"/>
-      <c r="M16" s="328" t="str">
+      <c r="D16" s="338" t="s">
+        <v>504</v>
+      </c>
+      <c r="E16" s="320">
+        <v>46268</v>
+      </c>
+      <c r="F16" s="321" t="s">
+        <v>505</v>
+      </c>
+      <c r="G16" s="322" t="s">
+        <v>506</v>
+      </c>
+      <c r="H16" s="323">
+        <v>9</v>
+      </c>
+      <c r="I16" s="324" t="s">
+        <v>507</v>
+      </c>
+      <c r="J16" s="325">
+        <v>4</v>
+      </c>
+      <c r="K16" s="326" t="s">
+        <v>508</v>
+      </c>
+      <c r="L16" s="327">
+        <v>7</v>
+      </c>
+      <c r="M16" s="328">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="N16" s="329" t="str">
+        <v>36</v>
+      </c>
+      <c r="N16" s="329">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="O16" s="318"/>
-      <c r="P16" s="330"/>
-      <c r="Q16" s="331"/>
-      <c r="R16" s="332"/>
-      <c r="S16" s="333"/>
-      <c r="T16" s="334"/>
-      <c r="U16" s="335" t="str">
+        <v>252</v>
+      </c>
+      <c r="O16" s="318" t="s">
+        <v>509</v>
+      </c>
+      <c r="P16" s="330" t="s">
+        <v>510</v>
+      </c>
+      <c r="Q16" s="331">
+        <v>46285</v>
+      </c>
+      <c r="R16" s="332">
+        <v>9</v>
+      </c>
+      <c r="S16" s="333">
+        <v>2</v>
+      </c>
+      <c r="T16" s="334">
+        <v>3</v>
+      </c>
+      <c r="U16" s="335">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="V16" s="329" t="str">
+        <v>18</v>
+      </c>
+      <c r="V16" s="329">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>54</v>
       </c>
       <c r="W16" s="336"/>
       <c r="X16" s="332"/>
@@ -40935,13 +40945,15 @@
       </c>
       <c r="AC16" s="335" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>Medium</v>
       </c>
       <c r="AD16" s="329" t="str">
         <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-      <c r="AE16" s="336"/>
+        <v>Medium</v>
+      </c>
+      <c r="AE16" s="336" t="s">
+        <v>511</v>
+      </c>
       <c r="AL16" s="81"/>
     </row>
     <row r="17" spans="2:38" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
@@ -42228,6 +42240,27 @@
     <row r="52" ht="35.1" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="AB1:AD1"/>
+    <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="AB2:AD2"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AB5:AD5"/>
+    <mergeCell ref="AC7:AD7"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="P9:P10"/>
+    <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="AD9:AD10"/>
     <mergeCell ref="AE9:AE10"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="X9:X10"/>
@@ -42244,27 +42277,6 @@
     <mergeCell ref="W9:W10"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="Z5:AA5"/>
-    <mergeCell ref="AB5:AD5"/>
-    <mergeCell ref="AC7:AD7"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="P9:P10"/>
-    <mergeCell ref="Q9:Q10"/>
-    <mergeCell ref="AD9:AD10"/>
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="AB1:AD1"/>
-    <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="AB2:AD2"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
   </mergeCells>
   <phoneticPr fontId="73" type="noConversion"/>
   <conditionalFormatting sqref="N11:N38">
@@ -42395,7 +42407,7 @@
     <row r="4" spans="2:14" ht="33" x14ac:dyDescent="0.35">
       <c r="B4" s="376">
         <f ca="1">TODAY()</f>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="C4" s="162"/>
       <c r="D4" s="162"/>
@@ -42944,13 +42956,13 @@
     <row r="1" spans="1:36" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="S1" s="5"/>
       <c r="Y1" s="5"/>
-      <c r="Z1" s="595" t="s">
+      <c r="Z1" s="550" t="s">
         <v>75</v>
       </c>
-      <c r="AA1" s="595"/>
-      <c r="AB1" s="595"/>
-      <c r="AC1" s="595"/>
-      <c r="AD1" s="595"/>
+      <c r="AA1" s="550"/>
+      <c r="AB1" s="550"/>
+      <c r="AC1" s="550"/>
+      <c r="AD1" s="550"/>
       <c r="AE1" s="2" t="s">
         <v>348</v>
       </c>
@@ -42963,22 +42975,22 @@
         <v>350</v>
       </c>
       <c r="S2" s="6"/>
-      <c r="T2" s="507" t="str">
+      <c r="T2" s="511" t="str">
         <f>"0 - "&amp;Y2</f>
         <v xml:space="preserve">0 - </v>
       </c>
-      <c r="U2" s="507"/>
+      <c r="U2" s="511"/>
       <c r="Y2" s="6"/>
-      <c r="Z2" s="507" t="str">
+      <c r="Z2" s="511" t="str">
         <f>"0 - "&amp;AE2</f>
         <v>0 - 249</v>
       </c>
-      <c r="AA2" s="507"/>
-      <c r="AB2" s="507" t="s">
+      <c r="AA2" s="511"/>
+      <c r="AB2" s="511" t="s">
         <v>351</v>
       </c>
-      <c r="AC2" s="507"/>
-      <c r="AD2" s="507"/>
+      <c r="AC2" s="511"/>
+      <c r="AD2" s="511"/>
       <c r="AE2" s="116">
         <v>249</v>
       </c>
@@ -42991,22 +43003,22 @@
         <v>292</v>
       </c>
       <c r="S3" s="6"/>
-      <c r="T3" s="508" t="str">
+      <c r="T3" s="512" t="str">
         <f>(Y2+1)&amp;" - "&amp;Y3</f>
         <v xml:space="preserve">1 - </v>
       </c>
-      <c r="U3" s="508"/>
+      <c r="U3" s="512"/>
       <c r="Y3" s="6"/>
-      <c r="Z3" s="508" t="str">
+      <c r="Z3" s="512" t="str">
         <f>(AE2+1)&amp;" - "&amp;AE3</f>
         <v>250 - 499</v>
       </c>
-      <c r="AA3" s="508"/>
-      <c r="AB3" s="508" t="s">
+      <c r="AA3" s="512"/>
+      <c r="AB3" s="512" t="s">
         <v>77</v>
       </c>
-      <c r="AC3" s="508"/>
-      <c r="AD3" s="508"/>
+      <c r="AC3" s="512"/>
+      <c r="AD3" s="512"/>
       <c r="AE3" s="116">
         <v>499</v>
       </c>
@@ -43021,41 +43033,41 @@
       <c r="D4" s="8"/>
       <c r="E4" s="9"/>
       <c r="F4" s="10"/>
-      <c r="G4" s="585" t="s">
+      <c r="G4" s="551" t="s">
         <v>353</v>
       </c>
-      <c r="H4" s="586"/>
-      <c r="I4" s="587"/>
+      <c r="H4" s="552"/>
+      <c r="I4" s="553"/>
       <c r="K4" s="11" t="s">
         <v>354</v>
       </c>
-      <c r="L4" s="591"/>
-      <c r="M4" s="591"/>
-      <c r="N4" s="591"/>
+      <c r="L4" s="557"/>
+      <c r="M4" s="557"/>
+      <c r="N4" s="557"/>
       <c r="O4" s="12"/>
       <c r="P4" s="13"/>
       <c r="Q4" s="14"/>
       <c r="R4" s="14"/>
       <c r="S4" s="6"/>
-      <c r="T4" s="592" t="str">
+      <c r="T4" s="558" t="str">
         <f>(Y3+1)&amp;" - "&amp;Y4</f>
         <v xml:space="preserve">1 - </v>
       </c>
-      <c r="U4" s="592"/>
+      <c r="U4" s="558"/>
       <c r="V4" s="14"/>
       <c r="W4" s="14"/>
       <c r="X4" s="14"/>
       <c r="Y4" s="6"/>
-      <c r="Z4" s="592" t="str">
+      <c r="Z4" s="558" t="str">
         <f>(AE3+1)&amp;" - "&amp;AE4</f>
         <v>500 - 749</v>
       </c>
-      <c r="AA4" s="592"/>
-      <c r="AB4" s="592" t="s">
+      <c r="AA4" s="558"/>
+      <c r="AB4" s="558" t="s">
         <v>355</v>
       </c>
-      <c r="AC4" s="592"/>
-      <c r="AD4" s="592"/>
+      <c r="AC4" s="558"/>
+      <c r="AD4" s="558"/>
       <c r="AE4" s="117">
         <v>749</v>
       </c>
@@ -43068,15 +43080,15 @@
       <c r="D5" s="16"/>
       <c r="E5" s="17"/>
       <c r="F5" s="18"/>
-      <c r="G5" s="588"/>
-      <c r="H5" s="589"/>
-      <c r="I5" s="590"/>
+      <c r="G5" s="554"/>
+      <c r="H5" s="555"/>
+      <c r="I5" s="556"/>
       <c r="K5" s="19" t="s">
         <v>356</v>
       </c>
-      <c r="L5" s="593"/>
-      <c r="M5" s="593"/>
-      <c r="N5" s="593"/>
+      <c r="L5" s="559"/>
+      <c r="M5" s="559"/>
+      <c r="N5" s="559"/>
       <c r="O5" s="20" t="s">
         <v>357</v>
       </c>
@@ -43084,25 +43096,25 @@
       <c r="Q5" s="22"/>
       <c r="R5" s="22"/>
       <c r="S5" s="6"/>
-      <c r="T5" s="594" t="str">
+      <c r="T5" s="560" t="str">
         <f>(Y4+1)&amp;" - "&amp;Y5</f>
         <v xml:space="preserve">1 - </v>
       </c>
-      <c r="U5" s="594"/>
+      <c r="U5" s="560"/>
       <c r="V5" s="22"/>
       <c r="W5" s="22"/>
       <c r="X5" s="22"/>
       <c r="Y5" s="6"/>
-      <c r="Z5" s="594" t="str">
+      <c r="Z5" s="560" t="str">
         <f>(AE4+1)&amp;" - "&amp;AE5</f>
         <v>750 - 1000</v>
       </c>
-      <c r="AA5" s="594"/>
-      <c r="AB5" s="594" t="s">
+      <c r="AA5" s="560"/>
+      <c r="AB5" s="560" t="s">
         <v>358</v>
       </c>
-      <c r="AC5" s="594"/>
-      <c r="AD5" s="594"/>
+      <c r="AC5" s="560"/>
+      <c r="AD5" s="560"/>
       <c r="AE5" s="117">
         <v>1000</v>
       </c>
@@ -43448,7 +43460,7 @@
       </c>
     </row>
     <row r="14" spans="1:36" s="60" customFormat="1" ht="112.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="569"/>
+      <c r="A14" s="563"/>
       <c r="B14" s="121"/>
       <c r="C14" s="122" t="s">
         <v>378</v>
@@ -43456,78 +43468,78 @@
       <c r="D14" s="123" t="s">
         <v>379</v>
       </c>
-      <c r="E14" s="571" t="s">
+      <c r="E14" s="565" t="s">
         <v>380</v>
       </c>
-      <c r="F14" s="573" t="s">
+      <c r="F14" s="567" t="s">
         <v>381</v>
       </c>
-      <c r="G14" s="575" t="s">
+      <c r="G14" s="569" t="s">
         <v>382</v>
       </c>
       <c r="H14" s="57" t="s">
         <v>383</v>
       </c>
-      <c r="I14" s="577" t="s">
+      <c r="I14" s="571" t="s">
         <v>384</v>
       </c>
       <c r="J14" s="58" t="s">
         <v>385</v>
       </c>
-      <c r="K14" s="579" t="s">
+      <c r="K14" s="573" t="s">
         <v>386</v>
       </c>
       <c r="L14" s="59" t="s">
         <v>387</v>
       </c>
-      <c r="M14" s="559" t="s">
+      <c r="M14" s="575" t="s">
         <v>388</v>
       </c>
-      <c r="N14" s="561" t="s">
+      <c r="N14" s="577" t="s">
         <v>389</v>
       </c>
-      <c r="O14" s="581" t="s">
+      <c r="O14" s="579" t="s">
         <v>390</v>
       </c>
-      <c r="P14" s="571" t="s">
+      <c r="P14" s="565" t="s">
         <v>391</v>
       </c>
-      <c r="Q14" s="583" t="s">
+      <c r="Q14" s="581" t="s">
         <v>392</v>
       </c>
-      <c r="R14" s="563" t="s">
+      <c r="R14" s="561" t="s">
         <v>393</v>
       </c>
-      <c r="S14" s="559" t="s">
+      <c r="S14" s="575" t="s">
         <v>385</v>
       </c>
-      <c r="T14" s="561" t="s">
+      <c r="T14" s="577" t="s">
         <v>387</v>
       </c>
-      <c r="U14" s="563" t="s">
+      <c r="U14" s="561" t="s">
         <v>388</v>
       </c>
-      <c r="V14" s="565"/>
-      <c r="W14" s="567" t="s">
+      <c r="V14" s="585"/>
+      <c r="W14" s="587" t="s">
         <v>394</v>
       </c>
-      <c r="X14" s="563" t="s">
+      <c r="X14" s="561" t="s">
         <v>393</v>
       </c>
-      <c r="Y14" s="559" t="s">
+      <c r="Y14" s="575" t="s">
         <v>385</v>
       </c>
-      <c r="Z14" s="561" t="s">
+      <c r="Z14" s="577" t="s">
         <v>387</v>
       </c>
-      <c r="AA14" s="563" t="s">
+      <c r="AA14" s="561" t="s">
         <v>388</v>
       </c>
-      <c r="AB14" s="565"/>
-      <c r="AC14" s="563" t="s">
+      <c r="AB14" s="585"/>
+      <c r="AC14" s="561" t="s">
         <v>395</v>
       </c>
-      <c r="AD14" s="557" t="s">
+      <c r="AD14" s="583" t="s">
         <v>396</v>
       </c>
       <c r="AE14" s="2"/>
@@ -43538,42 +43550,42 @@
       <c r="AJ14" s="2"/>
     </row>
     <row r="15" spans="1:36" s="60" customFormat="1" ht="53.25" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="570"/>
+      <c r="A15" s="564"/>
       <c r="B15" s="124"/>
       <c r="C15" s="125"/>
       <c r="D15" s="126"/>
-      <c r="E15" s="572"/>
-      <c r="F15" s="574"/>
-      <c r="G15" s="576"/>
+      <c r="E15" s="566"/>
+      <c r="F15" s="568"/>
+      <c r="G15" s="570"/>
       <c r="H15" s="61" t="s">
         <v>397</v>
       </c>
-      <c r="I15" s="578"/>
+      <c r="I15" s="572"/>
       <c r="J15" s="62" t="s">
         <v>397</v>
       </c>
-      <c r="K15" s="580"/>
+      <c r="K15" s="574"/>
       <c r="L15" s="62" t="s">
         <v>397</v>
       </c>
-      <c r="M15" s="560"/>
-      <c r="N15" s="562"/>
-      <c r="O15" s="582"/>
-      <c r="P15" s="572"/>
-      <c r="Q15" s="584"/>
-      <c r="R15" s="564"/>
-      <c r="S15" s="560"/>
-      <c r="T15" s="562"/>
-      <c r="U15" s="564"/>
-      <c r="V15" s="566"/>
-      <c r="W15" s="568"/>
-      <c r="X15" s="564"/>
-      <c r="Y15" s="560"/>
-      <c r="Z15" s="562"/>
-      <c r="AA15" s="564"/>
-      <c r="AB15" s="566"/>
-      <c r="AC15" s="564"/>
-      <c r="AD15" s="558"/>
+      <c r="M15" s="576"/>
+      <c r="N15" s="578"/>
+      <c r="O15" s="580"/>
+      <c r="P15" s="566"/>
+      <c r="Q15" s="582"/>
+      <c r="R15" s="562"/>
+      <c r="S15" s="576"/>
+      <c r="T15" s="578"/>
+      <c r="U15" s="562"/>
+      <c r="V15" s="586"/>
+      <c r="W15" s="588"/>
+      <c r="X15" s="562"/>
+      <c r="Y15" s="576"/>
+      <c r="Z15" s="578"/>
+      <c r="AA15" s="562"/>
+      <c r="AB15" s="586"/>
+      <c r="AC15" s="562"/>
+      <c r="AD15" s="584"/>
       <c r="AE15" s="2"/>
       <c r="AF15" s="2"/>
       <c r="AG15" s="2"/>
@@ -43585,10 +43597,10 @@
       <c r="A16" s="127" t="s">
         <v>398</v>
       </c>
-      <c r="B16" s="550" t="s">
+      <c r="B16" s="589" t="s">
         <v>399</v>
       </c>
-      <c r="C16" s="553" t="s">
+      <c r="C16" s="592" t="s">
         <v>400</v>
       </c>
       <c r="D16" s="128" t="s">
@@ -43673,8 +43685,8 @@
       <c r="A17" s="63" t="s">
         <v>402</v>
       </c>
-      <c r="B17" s="551"/>
-      <c r="C17" s="554"/>
+      <c r="B17" s="590"/>
+      <c r="C17" s="593"/>
       <c r="D17" s="143" t="s">
         <v>403</v>
       </c>
@@ -43757,8 +43769,8 @@
       <c r="A18" s="63" t="s">
         <v>404</v>
       </c>
-      <c r="B18" s="551"/>
-      <c r="C18" s="555"/>
+      <c r="B18" s="590"/>
+      <c r="C18" s="594"/>
       <c r="D18" s="143" t="s">
         <v>405</v>
       </c>
@@ -43839,7 +43851,7 @@
       <c r="A19" s="63" t="s">
         <v>406</v>
       </c>
-      <c r="B19" s="551"/>
+      <c r="B19" s="590"/>
       <c r="C19" s="73" t="s">
         <v>407</v>
       </c>
@@ -43922,8 +43934,8 @@
       <c r="A20" s="63" t="s">
         <v>408</v>
       </c>
-      <c r="B20" s="551"/>
-      <c r="C20" s="556" t="s">
+      <c r="B20" s="590"/>
+      <c r="C20" s="595" t="s">
         <v>409</v>
       </c>
       <c r="D20" s="143" t="s">
@@ -43988,8 +44000,8 @@
       <c r="A21" s="63" t="s">
         <v>410</v>
       </c>
-      <c r="B21" s="552"/>
-      <c r="C21" s="555"/>
+      <c r="B21" s="591"/>
+      <c r="C21" s="594"/>
       <c r="D21" s="143" t="s">
         <v>403</v>
       </c>
@@ -44052,10 +44064,10 @@
       <c r="A22" s="63" t="s">
         <v>411</v>
       </c>
-      <c r="B22" s="550" t="s">
+      <c r="B22" s="589" t="s">
         <v>412</v>
       </c>
-      <c r="C22" s="553" t="s">
+      <c r="C22" s="592" t="s">
         <v>400</v>
       </c>
       <c r="D22" s="128" t="s">
@@ -44120,8 +44132,8 @@
       <c r="A23" s="63" t="s">
         <v>413</v>
       </c>
-      <c r="B23" s="551"/>
-      <c r="C23" s="554"/>
+      <c r="B23" s="590"/>
+      <c r="C23" s="593"/>
       <c r="D23" s="143" t="s">
         <v>403</v>
       </c>
@@ -44184,8 +44196,8 @@
       <c r="A24" s="63" t="s">
         <v>414</v>
       </c>
-      <c r="B24" s="551"/>
-      <c r="C24" s="555"/>
+      <c r="B24" s="590"/>
+      <c r="C24" s="594"/>
       <c r="D24" s="143" t="s">
         <v>405</v>
       </c>
@@ -44248,7 +44260,7 @@
       <c r="A25" s="63" t="s">
         <v>415</v>
       </c>
-      <c r="B25" s="551"/>
+      <c r="B25" s="590"/>
       <c r="C25" s="73" t="s">
         <v>407</v>
       </c>
@@ -44314,8 +44326,8 @@
       <c r="A26" s="63" t="s">
         <v>416</v>
       </c>
-      <c r="B26" s="551"/>
-      <c r="C26" s="556" t="s">
+      <c r="B26" s="590"/>
+      <c r="C26" s="595" t="s">
         <v>409</v>
       </c>
       <c r="D26" s="143" t="s">
@@ -44380,8 +44392,8 @@
       <c r="A27" s="63" t="s">
         <v>417</v>
       </c>
-      <c r="B27" s="552"/>
-      <c r="C27" s="555"/>
+      <c r="B27" s="591"/>
+      <c r="C27" s="594"/>
       <c r="D27" s="143" t="s">
         <v>403</v>
       </c>
@@ -45352,22 +45364,24 @@
     <row r="56" spans="38:38" ht="35.1" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="Z1:AD1"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="AB2:AD2"/>
-    <mergeCell ref="T3:U3"/>
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="AB3:AD3"/>
-    <mergeCell ref="G4:I5"/>
-    <mergeCell ref="L4:N4"/>
-    <mergeCell ref="T4:U4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="T5:U5"/>
-    <mergeCell ref="Z5:AA5"/>
-    <mergeCell ref="AB5:AD5"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="B22:B27"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="AD14:AD15"/>
+    <mergeCell ref="S14:S15"/>
+    <mergeCell ref="T14:T15"/>
+    <mergeCell ref="U14:U15"/>
+    <mergeCell ref="V14:V15"/>
+    <mergeCell ref="W14:W15"/>
+    <mergeCell ref="X14:X15"/>
+    <mergeCell ref="Y14:Y15"/>
+    <mergeCell ref="Z14:Z15"/>
+    <mergeCell ref="AA14:AA15"/>
+    <mergeCell ref="AB14:AB15"/>
+    <mergeCell ref="AC14:AC15"/>
     <mergeCell ref="R14:R15"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="E14:E15"/>
@@ -45380,24 +45394,22 @@
     <mergeCell ref="O14:O15"/>
     <mergeCell ref="P14:P15"/>
     <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="AD14:AD15"/>
-    <mergeCell ref="S14:S15"/>
-    <mergeCell ref="T14:T15"/>
-    <mergeCell ref="U14:U15"/>
-    <mergeCell ref="V14:V15"/>
-    <mergeCell ref="W14:W15"/>
-    <mergeCell ref="X14:X15"/>
-    <mergeCell ref="Y14:Y15"/>
-    <mergeCell ref="Z14:Z15"/>
-    <mergeCell ref="AA14:AA15"/>
-    <mergeCell ref="AB14:AB15"/>
-    <mergeCell ref="AC14:AC15"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="B22:B27"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="G4:I5"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="Z5:AA5"/>
+    <mergeCell ref="AB5:AD5"/>
+    <mergeCell ref="Z1:AD1"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="AB2:AD2"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="AB3:AD3"/>
   </mergeCells>
   <conditionalFormatting sqref="N16:N42">
     <cfRule type="cellIs" dxfId="22" priority="6" stopIfTrue="1" operator="equal">
@@ -45672,15 +45684,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="488869cc-a9d1-4445-93a6-e9d986f2ee4c">
@@ -45688,6 +45691,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -45709,14 +45721,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64B48805-C4FD-4969-846E-6B980EB12FDA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{949992B3-0D0A-42A8-9229-662793BD027C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -45724,4 +45728,12 @@
     <ds:schemaRef ds:uri="488869cc-a9d1-4445-93a6-e9d986f2ee4c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64B48805-C4FD-4969-846E-6B980EB12FDA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>